<commit_message>
docs: update README for handover, remove internal tooling references
- Rewrote README with full framework documentation: architecture,
  test counts, per-country breakdown, setup instructions, and
  maintenance guide
- Removed internal development configuration files
- Updated .gitignore to exclude temporary files

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Order_Engine_Test_Inventory.xlsx
+++ b/Order_Engine_Test_Inventory.xlsx
@@ -10475,7 +10475,7 @@
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10500,7 +10500,7 @@
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10525,7 +10525,7 @@
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10550,7 +10550,7 @@
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10575,7 +10575,7 @@
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10600,7 +10600,7 @@
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10625,7 +10625,7 @@
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10650,7 +10650,7 @@
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10675,7 +10675,7 @@
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10700,7 +10700,7 @@
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10725,7 +10725,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10750,7 +10750,7 @@
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10775,7 +10775,7 @@
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10800,7 +10800,7 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10825,7 +10825,7 @@
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10850,7 +10850,7 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10875,7 +10875,7 @@
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10900,7 +10900,7 @@
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10925,7 +10925,7 @@
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10950,7 +10950,7 @@
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -10975,7 +10975,7 @@
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -11000,7 +11000,7 @@
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -11025,7 +11025,7 @@
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -11050,7 +11050,7 @@
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -11075,7 +11075,7 @@
       </c>
       <c r="E108" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -11100,7 +11100,7 @@
       </c>
       <c r="E109" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -11125,7 +11125,7 @@
       </c>
       <c r="E110" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -11150,7 +11150,7 @@
       </c>
       <c r="E111" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -11175,7 +11175,7 @@
       </c>
       <c r="E112" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>
@@ -11200,7 +11200,7 @@
       </c>
       <c r="E113" s="3" t="inlineStr">
         <is>
-          <t>Sub-step of France Postcode Checker (Excel IDs 443322/443323)</t>
+          <t>Sub-step of France Postcode Checker (Excel 443322/443323)</t>
         </is>
       </c>
     </row>

</xml_diff>